<commit_message>
feat: Make QuantityValue.numeric_value optional and add 'collected' status
This commit makes two important schema changes to better support real-world
experimental data:

1. **Make QuantityValue.numeric_value optional**: Changed from required to
   optional to allow for cases where measurements are unknown, not applicable,
   or not yet recorded. This is common in experimental data where some
   parameters may not be measured or recorded.

2. **Add 'collected' to ProcessingStatusEnum**: Added a new status value
   'collected' to represent data that has been collected but not yet processed.
   This fills a gap in the status progression and matches common terminology
   in experimental workflows.

These changes address validation issues in PR #69 where real-world data from
NSLS-II AMX beamline included null values for some measurements and used
'collected' as a processing status.

Fixes #69

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -2866,7 +2866,7 @@
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography"</formula1>
+      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"synchrotron,rotating_anode,microfocus,metal_jet"</formula1>
@@ -3240,13 +3240,13 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography"</formula1>
+      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x_ray_diffraction,neutron_diffraction,electron_diffraction,fiber_diffraction"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"raw,preprocessing,processing,completed,failed"</formula1>
+      <formula1>"collected,raw,preprocessing,processing,completed,failed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: resolve merge conflicts and regenerate assets
- Resolve NCBITaxon prefix conflicts (use uppercase per convention)
- Remove duplicate prefix entries (simplescattering, pdb)
- Regenerate all assets from schema

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -1596,7 +1596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG1"/>
+  <dimension ref="A1:AH1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1752,15 +1752,20 @@
       </c>
       <c r="AE1" t="inlineStr">
         <is>
+          <t>oligomeric_state</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3725,7 +3730,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"mrc,tiff,hdf5,star,pdb,mmcif,mtz,cbf,cbf_zst,img,h5,ascii,thermo_raw,zip,mrcs,eer,cs,json,csv,ccp4,gz"</formula1>
+      <formula1>"mrc,tiff,hdf5,star,pdb,mmcif,mtz,cbf,cbf_zst,img,h5,ascii,thermo_raw,zip,tar,mrcs,eer,cs,json,csv,ccp4,gz"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"micrograph,diffraction,scattering,particles,volume,model,metadata,raw_data,processed_data,movie,motion_corrected,ctf_estimation,particle_coordinates,class_averages,fsc_curve,map_half,validation_report"</formula1>

</xml_diff>

<commit_message>
Update schema artifacts, including docs
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -63,21 +63,22 @@
     <sheet name="SAXSPreparation" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="ExperimentalConditions" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="DataCollectionStrategy" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="QualityMetrics" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="ComputeResources" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="MotionCorrectionParameters" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="CTFEstimationParameters" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="ParticlePickingParameters" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="RefinementParameters" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="FSCCurve" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="StudySampleAssociation" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="StudyExperimentAssociation" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="StudyWorkflowAssociation" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="ExperimentSampleAssociation" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="ExperimentInstrumentAssociation" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="WorkflowExperimentAssociation" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="WorkflowInputAssociation" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="WorkflowOutputAssociation" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="BeamCenterPixels" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="QualityMetrics" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="ComputeResources" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="MotionCorrectionParameters" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="CTFEstimationParameters" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="ParticlePickingParameters" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="RefinementParameters" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="FSCCurve" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="StudySampleAssociation" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="StudyExperimentAssociation" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="StudyWorkflowAssociation" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="ExperimentSampleAssociation" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="ExperimentInstrumentAssociation" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="WorkflowExperimentAssociation" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="WorkflowInputAssociation" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="WorkflowOutputAssociation" sheetId="72" state="visible" r:id="rId72"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3308,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG1"/>
+  <dimension ref="A1:BL1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3469,140 +3470,165 @@
       </c>
       <c r="AF1" t="inlineStr">
         <is>
+          <t>detector</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
           <t>wavelength</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>energy</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
         <is>
           <t>oscillation_angle</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>start_angle</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>sweep_start</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>sweep_end</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
         <is>
           <t>number_of_images</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>beam_center_x</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>beam_center_y</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>beam_center_pixels</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>detector_distance</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>pixel_size_x</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>pixel_size_y</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>total_rotation</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>beamline</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>transmission</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>flux</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>flux_end</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>slit_gap_horizontal</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>slit_gap_vertical</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>undulator_gap</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>synchrotron_mode</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>exposure_time</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>start_time</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>end_time</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>resolution</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>resolution_at_corner</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>ispyb_data_collection_id</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>ispyb_session_id</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -5758,7 +5784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5819,45 +5845,70 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>beam_center_pixels</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>beam_size_um</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>energy</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>flux_photons_per_s</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>transmission_percent</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>attenuator</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>temperature_k</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>oscillation_per_image_deg</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>sweep_start</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>sweep_end</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
         <is>
           <t>total_rotation_deg</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
         <is>
           <t>strategy_notes</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -5877,6 +5928,37 @@
 </file>
 
 <file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>xbeam</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ybeam</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6057,7 +6139,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6088,67 +6170,6 @@
         </is>
       </c>
       <c r="E1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>patch_size</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>binning</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>dose_weighting</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>bfactor_dose_weighting</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>anisotropic_correction</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>frame_grouping</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>output_binning</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>drift_total</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -6251,41 +6272,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>defocus_search_min</t>
+          <t>patch_size</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>defocus_search_max</t>
+          <t>binning</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>defocus_step</t>
+          <t>dose_weighting</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>amplitude_contrast</t>
+          <t>bfactor_dose_weighting</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>cs_used_in_estimation</t>
+          <t>anisotropic_correction</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>voltage_used_in_estimation</t>
+          <t>frame_grouping</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
+        <is>
+          <t>output_binning</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>drift_total</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -6302,51 +6333,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>picking_method</t>
+          <t>defocus_search_min</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>box_size</t>
+          <t>defocus_search_max</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>threshold</t>
+          <t>defocus_step</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>power_score</t>
+          <t>amplitude_contrast</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>ncc_score</t>
+          <t>cs_used_in_estimation</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>model_name</t>
+          <t>voltage_used_in_estimation</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>model_file_path</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>model_source</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -6369,6 +6390,67 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>picking_method</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>box_size</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>threshold</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>power_score</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ncc_score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>model_name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>model_file_path</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>model_source</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>symmetry</t>
         </is>
       </c>
@@ -6423,7 +6505,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6454,7 +6536,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6491,32 +6573,6 @@
       <formula1>"target,control,reference,blank"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>study_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>experiment_id</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6538,7 +6594,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>workflow_id</t>
+          <t>experiment_id</t>
         </is>
       </c>
     </row>
@@ -6548,6 +6604,32 @@
 </file>
 
 <file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>study_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>workflow_id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6588,7 +6670,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6620,32 +6702,6 @@
       <formula1>"primary,detector,sample_handler"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>workflow_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>experiment_id</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6782,7 +6838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6793,21 +6849,11 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>file_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>input_type</t>
+          <t>experiment_id</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"raw_data,reference,parameters,mask"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6834,6 +6880,42 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>input_type</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"raw_data,reference,parameters,mask"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>workflow_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>file_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>output_type</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Regenerate assets from schema
Rebuild downstream artifacts (JSON Schema, Python, OWL, SHACL, GraphQL,
JSON-LD, Protobuf, SQL, Excel, prefixmap) via `make gen-project` to reflect
the new instrument_registry_id slot, the added BeamlineEnum entries, and the
removed ExperimentRun.beamline slot. Markdown docs are excluded from
gen-project (built separately into docs/elements via `make gendoc`).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -2180,7 +2180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2191,55 +2191,60 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>instrument_registry_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2247,13 +2252,13 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2267,7 +2272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL1"/>
+  <dimension ref="A1:AM1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2408,55 +2413,60 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>instrument_registry_id</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2473,13 +2483,13 @@
     <dataValidation sqref="Y2:Y1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"EFTEM,TEM,STEM"</formula1>
     </dataValidation>
-    <dataValidation sqref="AB2:AB1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AC2:AC1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="AC2:AC1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AD2:AD1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="AI2:AI1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AJ2:AJ1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2493,7 +2503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2564,55 +2574,60 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>instrument_registry_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2626,13 +2641,13 @@
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"direct_electron_detector,ccd,cmos,hybrid_photon_counting,scintillator_coupled,imaging_plate,film"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="V2:V1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2905,7 +2920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2951,55 +2966,60 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>instrument_registry_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3010,13 +3030,13 @@
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3030,7 +3050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3071,55 +3091,60 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>instrument_registry_id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3127,13 +3152,13 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3147,7 +3172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3218,55 +3243,60 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>instrument_registry_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3289,13 +3319,13 @@
     <dataValidation sqref="L2:L1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"epics,tango,labview,opi"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="V2:V1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3309,7 +3339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL1"/>
+  <dimension ref="A1:BK1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3545,90 +3575,85 @@
       </c>
       <c r="AU1" t="inlineStr">
         <is>
-          <t>beamline</t>
+          <t>transmission</t>
         </is>
       </c>
       <c r="AV1" t="inlineStr">
         <is>
-          <t>transmission</t>
+          <t>flux</t>
         </is>
       </c>
       <c r="AW1" t="inlineStr">
         <is>
-          <t>flux</t>
+          <t>flux_end</t>
         </is>
       </c>
       <c r="AX1" t="inlineStr">
         <is>
-          <t>flux_end</t>
+          <t>slit_gap_horizontal</t>
         </is>
       </c>
       <c r="AY1" t="inlineStr">
         <is>
-          <t>slit_gap_horizontal</t>
+          <t>slit_gap_vertical</t>
         </is>
       </c>
       <c r="AZ1" t="inlineStr">
         <is>
-          <t>slit_gap_vertical</t>
+          <t>undulator_gap</t>
         </is>
       </c>
       <c r="BA1" t="inlineStr">
         <is>
-          <t>undulator_gap</t>
+          <t>synchrotron_mode</t>
         </is>
       </c>
       <c r="BB1" t="inlineStr">
         <is>
-          <t>synchrotron_mode</t>
+          <t>exposure_time</t>
         </is>
       </c>
       <c r="BC1" t="inlineStr">
         <is>
-          <t>exposure_time</t>
+          <t>start_time</t>
         </is>
       </c>
       <c r="BD1" t="inlineStr">
         <is>
-          <t>start_time</t>
+          <t>end_time</t>
         </is>
       </c>
       <c r="BE1" t="inlineStr">
         <is>
-          <t>end_time</t>
+          <t>resolution</t>
         </is>
       </c>
       <c r="BF1" t="inlineStr">
         <is>
-          <t>resolution</t>
+          <t>resolution_at_corner</t>
         </is>
       </c>
       <c r="BG1" t="inlineStr">
         <is>
-          <t>resolution_at_corner</t>
+          <t>ispyb_data_collection_id</t>
         </is>
       </c>
       <c r="BH1" t="inlineStr">
         <is>
-          <t>ispyb_data_collection_id</t>
+          <t>ispyb_session_id</t>
         </is>
       </c>
       <c r="BI1" t="inlineStr">
         <is>
-          <t>ispyb_session_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="BJ1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>title</t>
         </is>
       </c>
       <c r="BK1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="BL1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Regenerate pydantic model, assets, docs, and examples
The schema additions in this branch never propagated to the generated
artifacts, so the package's own Python API rejected every new feature:
Study(proposal_id=...) raised a validation error under extra="forbid",
TechniqueEnum.microed did not exist, and CryoEMQualityMetrics could not
be imported. The shipped JSON Schema likewise had Study with
additionalProperties: false and no proposal_id, which meant this branch's
own Study-proposal-id.yaml fixture failed against it.

Runs `make all` and commits the result: pydantic.py, assets/, docs/, and
the example renders. Also picks up the docs backlog for
instrument_registry_id from #110.

Note that CI does not regenerate assets/ -- only docs/ is rebuilt at
deploy time -- so this drift is not caught automatically.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -66,19 +66,20 @@
     <sheet name="BeamCenterPixels" sheetId="57" state="visible" r:id="rId57"/>
     <sheet name="QualityMetrics" sheetId="58" state="visible" r:id="rId58"/>
     <sheet name="ComputeResources" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="MotionCorrectionParameters" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="CTFEstimationParameters" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="ParticlePickingParameters" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="RefinementParameters" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="FSCCurve" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="StudySampleAssociation" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="StudyExperimentAssociation" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="StudyWorkflowAssociation" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="ExperimentSampleAssociation" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="ExperimentInstrumentAssociation" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="WorkflowExperimentAssociation" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="WorkflowInputAssociation" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="WorkflowOutputAssociation" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="CryoEMQualityMetrics" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="MotionCorrectionParameters" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="CTFEstimationParameters" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="ParticlePickingParameters" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="RefinementParameters" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="FSCCurve" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="StudySampleAssociation" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="StudyExperimentAssociation" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="StudyWorkflowAssociation" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="ExperimentSampleAssociation" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="ExperimentInstrumentAssociation" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="WorkflowExperimentAssociation" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="WorkflowInputAssociation" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="WorkflowOutputAssociation" sheetId="73" state="visible" r:id="rId73"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1565,26 +1566,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>proposal_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>keywords</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3028,7 +3034,7 @@
   </sheetData>
   <dataValidations count="4">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography"</formula1>
+      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography,microed"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
@@ -3305,7 +3311,7 @@
   </sheetData>
   <dataValidations count="8">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography"</formula1>
+      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography,microed"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"synchrotron,rotating_anode,microfocus,metal_jet"</formula1>
@@ -3339,7 +3345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK1"/>
+  <dimension ref="A1:BW1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3475,194 +3481,254 @@
       </c>
       <c r="AA1" t="inlineStr">
         <is>
+          <t>tilting_scheme</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>tilt_angle_min</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>tilt_angle_max</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>tilt_angle_increment</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>tilt_axis_angle</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>number_of_tilt_images</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>dose_per_tilt</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>dual_tilt_axis_rotation</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>fiducial_size</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>rotation_rate</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>camera_length</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>frames_per_second</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
           <t>autoloader_slot</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>shots_per_hole</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>holes_per_group</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>acquisition_software</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>acquisition_software_version</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>detector</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>wavelength</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>energy</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>oscillation_angle</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>start_angle</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>sweep_start</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>sweep_end</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>number_of_images</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>beam_center_x</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>beam_center_y</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>beam_center_pixels</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>detector_distance</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>pixel_size_x</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>pixel_size_y</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>total_rotation</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>transmission</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>flux</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>flux_end</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>slit_gap_horizontal</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>slit_gap_vertical</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>undulator_gap</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>synchrotron_mode</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>exposure_time</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>start_time</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>end_time</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>resolution</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>resolution_at_corner</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>ispyb_data_collection_id</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>ispyb_session_id</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography"</formula1>
+      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography,microed"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x_ray_diffraction,neutron_diffraction,electron_diffraction,fiber_diffraction"</formula1>
@@ -3672,6 +3738,9 @@
     </dataValidation>
     <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"bluesky,spec,sardana,gda,mxcube_daq,blu_ice,jblue_ice"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA2:AA1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"none,dose_symmetric,linear,continuous"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5989,7 +6058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG1"/>
+  <dimension ref="A1:AH1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6150,10 +6219,15 @@
       </c>
       <c r="AF1" t="inlineStr">
         <is>
+          <t>cryo_em</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
           <t>r_factor</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -6297,6 +6371,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ice_contamination</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ice_quality</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>particle_concentration</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"none,limited,severe"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ideal,too_thin,too_thick"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"optimal,too_low,too_high"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -6352,7 +6473,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6393,67 +6514,6 @@
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>picking_method</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>box_size</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>threshold</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>power_score</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>ncc_score</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>model_name</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>model_file_path</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>model_source</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -6476,6 +6536,67 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>picking_method</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>box_size</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>threshold</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>power_score</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ncc_score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>model_name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>model_file_path</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>model_source</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>symmetry</t>
         </is>
       </c>
@@ -6530,7 +6651,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6561,7 +6682,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6598,32 +6719,6 @@
       <formula1>"target,control,reference,blank"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>study_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>experiment_id</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6645,7 +6740,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>workflow_id</t>
+          <t>experiment_id</t>
         </is>
       </c>
     </row>
@@ -6655,6 +6750,32 @@
 </file>
 
 <file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>study_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>workflow_id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6689,42 +6810,6 @@
   <dataValidations count="1">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"target,buffer_blank,standard,size_marker"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>experiment_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>instrument_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"primary,detector,sample_handler"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6863,22 +6948,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>workflow_id</t>
+          <t>experiment_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>experiment_id</t>
+          <t>instrument_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>role</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"primary,detector,sample_handler"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6889,7 +6984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6900,21 +6995,11 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>file_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>input_type</t>
+          <t>experiment_id</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"raw_data,reference,parameters,mask"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6941,6 +7026,42 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>input_type</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"raw_data,reference,parameters,mask"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>workflow_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>file_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>output_type</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Regenerate artifacts for the Person, Organization and profile additions
make gen-project and make gen-rocrate. Person, Organization and their
association tables propagate into the JSON Schema, OWL, SHACL, SQL DDL, GraphQL,
Protobuf and Python artifacts; the SQL projection keeps the self-referential
parent_organization_id foreign key. assets/rocrate holds the profile's own
generated JSON Schema, JSON-LD context, OWL, prefix map and SSSOM crosswalk.

The crosswalk is the artifact that matters most here: it carries every crate
term to its schema slot, including the deprecated SSRL 0.2 spellings and the
parallel SAXS profile's, so migration is a lookup rather than prose someone has
to transcribe. Note that deprecated_element_has_exact_replacement is
documentation and not a mapping predicate gen-sssom reads, which is why each
deprecated term also carries an explicit mapping to its replacement.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -28,57 +28,64 @@
     <sheet name="MeasurementConditions" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Dataset" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="Study" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Sample" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="ProteinConstruct" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="SamplePreparation" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Instrument" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="CryoEMInstrument" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="XRayInstrument" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="SANSDetector" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="SANSSource" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="SANSConfiguration" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="SANSInstrument" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="SAXSInstrument" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="BeamlineInstrument" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="ExperimentRun" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="WorkflowRun" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="DataFile" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="Image" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="Image2D" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="Image3D" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="Movie" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="Micrograph" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="FTIRImage" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="FluorescenceImage" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="OpticalImage" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="XRFImage" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="ImageFeature" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="OntologyTerm" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="MolecularComposition" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="BufferComposition" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="StorageConditions" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="CryoEMPreparation" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="CrystallizationConditions" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="XRayPreparation" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="SAXSPreparation" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="ExperimentalConditions" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="DataCollectionStrategy" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="BeamCenterPixels" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="QualityMetrics" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="ComputeResources" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="MotionCorrectionParameters" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="CTFEstimationParameters" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="ParticlePickingParameters" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="RefinementParameters" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="FSCCurve" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="StudySampleAssociation" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="StudyExperimentAssociation" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="StudyWorkflowAssociation" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="ExperimentSampleAssociation" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="ExperimentInstrumentAssociation" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="WorkflowExperimentAssociation" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="WorkflowInputAssociation" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="WorkflowOutputAssociation" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="Person" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Organization" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Sample" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="ProteinConstruct" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="SamplePreparation" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Instrument" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="CryoEMInstrument" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="XRayInstrument" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="SANSDetector" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="SANSSource" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="SANSConfiguration" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="SANSInstrument" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="SAXSInstrument" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="BeamlineInstrument" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="ExperimentRun" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="WorkflowRun" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="DataFile" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="Image" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="Image2D" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="Image3D" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="Movie" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="Micrograph" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="FTIRImage" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="FluorescenceImage" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="OpticalImage" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="XRFImage" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="ImageFeature" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="OntologyTerm" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="MolecularComposition" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="BufferComposition" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="StorageConditions" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="CryoEMPreparation" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="CrystallizationConditions" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="XRayPreparation" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="SAXSPreparation" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="ExperimentalConditions" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="DataCollectionStrategy" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="BeamCenterPixels" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="QualityMetrics" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="ComputeResources" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="MotionCorrectionParameters" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="CTFEstimationParameters" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="ParticlePickingParameters" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="RefinementParameters" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="FSCCurve" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="StudySampleAssociation" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="StudyExperimentAssociation" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="StudyWorkflowAssociation" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="ExperimentSampleAssociation" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="ExperimentInstrumentAssociation" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="WorkflowExperimentAssociation" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="WorkflowInputAssociation" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="WorkflowOutputAssociation" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="StudyPersonAssociation" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="ExperimentPersonAssociation" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="WorkflowPersonAssociation" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="StudyOrganizationAssociation" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="PersonOrganizationAssociation" sheetId="79" state="visible" r:id="rId79"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1444,7 +1451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1460,142 +1467,350 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>organizations</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>instruments</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>protein_constructs</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>samples</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>sample_preparations</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>experiment_runs</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>workflow_runs</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>data_files</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>study_sample_associations</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>study_experiment_associations</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>study_workflow_associations</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>experiment_sample_associations</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>experiment_instrument_associations</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>workflow_experiment_associations</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>workflow_input_associations</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>workflow_output_associations</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>study_person_associations</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>experiment_person_associations</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>workflow_person_associations</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>study_organization_associations</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>person_organization_associations</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>keywords</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>protein_constructs</t>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>full_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>given_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>family_name</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>samples</t>
+          <t>email</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>sample_preparations</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>experiment_runs</t>
+          <t>affiliation_ror</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>workflow_runs</t>
+          <t>person_local_id</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>data_files</t>
+          <t>id</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>title</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>study_sample_associations</t>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ror</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>acronym</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>organization_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>facility_code</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>facility_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>parent_organization_id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>wikidata_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>is_doe_facility</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>study_experiment_associations</t>
+          <t>doe_office</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>study_workflow_associations</t>
+          <t>id</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>experiment_sample_associations</t>
+          <t>title</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>experiment_instrument_associations</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>workflow_experiment_associations</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>workflow_input_associations</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>workflow_output_associations</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
           <t>description</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>keywords</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+  <dataValidations count="3">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"national_laboratory,university,research_institute,government_agency,funding_agency,company,hospital,consortium,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SYNCHROTRON,NEUTRON_SOURCE,FREE_ELECTRON_LASER,CRYOEM_CENTER"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1786,7 +2001,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1922,7 +2137,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2174,13 +2389,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2211,40 +2426,45 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>facility_organization_id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2258,7 +2478,7 @@
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2266,13 +2486,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AM1"/>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AN1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2433,40 +2653,45 @@
       </c>
       <c r="AF1" t="inlineStr">
         <is>
+          <t>facility_organization_id</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2489,7 +2714,7 @@
     <dataValidation sqref="AD2:AD1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="AJ2:AJ1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AK2:AK1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2497,13 +2722,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Y1"/>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2594,40 +2819,45 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>facility_organization_id</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2647,7 +2877,7 @@
     <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="W2:W1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2655,7 +2885,58 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>maximum_numeric_value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>minimum_numeric_value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>numeric_value</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>unit_cv_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2726,7 +3007,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2782,244 +3063,198 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>maximum_numeric_value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>minimum_numeric_value</t>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>q_min</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>q_max</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>numeric_value</t>
+          <t>number_of_guides</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>attenuator</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>unit_cv_id</t>
+          <t>source_aperature_diameter</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>attribute</t>
+          <t>sample_aperature_diameter</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>q_min</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>q_max</t>
+          <t>siwindow_to_main_distance</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>sample_ap_to_si_distance</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>sample_ap_to_main_distance</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>sample_ap_to_sample_distance</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>source_ap_to_siwindow_distance</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>source_ap_to_sample_ap_distance</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>technique</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>q_range_min</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>number_of_guides</t>
+          <t>q_range_max</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>attenuator</t>
+          <t>detectors</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>source_aperature_diameter</t>
+          <t>source</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>sample_aperature_diameter</t>
+          <t>configuration</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>siwindow_to_main_distance</t>
+          <t>environment</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>sample_ap_to_si_distance</t>
+          <t>instrument_code</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>sample_ap_to_main_distance</t>
+          <t>instrument_registry_id</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>sample_ap_to_sample_distance</t>
+          <t>instrument_category</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>source_ap_to_siwindow_distance</t>
+          <t>facility_name</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>source_ap_to_sample_ap_distance</t>
+          <t>facility_ror</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:T1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>technique</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>q_range_min</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>q_range_max</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>detectors</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>configuration</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>environment</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>instrument_code</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>instrument_registry_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>instrument_category</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>facility_name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>facility_ror</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
+          <t>facility_organization_id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3036,7 +3271,7 @@
     <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="R2:R1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3044,13 +3279,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:S1"/>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3111,40 +3346,45 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>facility_organization_id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3158,7 +3398,7 @@
     <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3166,13 +3406,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Y1"/>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3263,40 +3503,45 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>facility_organization_id</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3325,7 +3570,7 @@
     <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="W2:W1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3333,7 +3578,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3678,7 +3923,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4039,7 +4284,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4128,7 +4373,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4194,7 +4439,43 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value_cv_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4270,7 +4551,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4351,184 +4632,476 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>value_cv_id</t>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AA1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>frames</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>super_resolution</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>attribute</t>
+          <t>pixel_size_unbinned</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AA1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>frames</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>super_resolution</t>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>stage_position_x</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>stage_position_y</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>stage_position_z</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>nominal_defocus</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>dose_per_frame</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>beam_shift_x</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>beam_shift_y</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ice_thickness_estimate</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>grid_square_id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>hole_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>acquisition_group</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>defocus</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>astigmatism</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>origin_movie_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>pixel_size_unbinned</t>
+          <t>defocus_u</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>defocus_v</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>stage_position_x</t>
+          <t>astigmatism_angle</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>stage_position_y</t>
+          <t>resolution_fit_limit</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>stage_position_z</t>
+          <t>ctf_quality_score</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>nominal_defocus</t>
+          <t>defocus</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>dose_per_frame</t>
+          <t>astigmatism</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>beam_shift_x</t>
+          <t>file_name</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>beam_shift_y</t>
+          <t>acquisition_date</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>ice_thickness_estimate</t>
+          <t>pixel_size</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>grid_square_id</t>
+          <t>dimensions_x</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>hole_id</t>
+          <t>dimensions_y</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>acquisition_group</t>
+          <t>exposure_time</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>wavenumber_min</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>wavenumber_max</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>spectral_resolution</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>number_of_scans</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>apodization_function</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>molecular_signatures</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>background_correction</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>excitation_wavelength</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>emission_wavelength</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>excitation_filter</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>emission_filter</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fluorophore</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>channel_name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>laser_power</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>pinhole_size</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>quantum_yield</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>defocus</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>astigmatism</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>astigmatism</t>
+          <t>exposure_time</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>file_name</t>
+          <t>dose</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>acquisition_date</t>
+          <t>id</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>pixel_size</t>
+          <t>title</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
           <t>description</t>
         </is>
       </c>
@@ -4538,335 +5111,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:R1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>origin_movie_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>defocus_u</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>defocus_v</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>astigmatism_angle</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>resolution_fit_limit</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>ctf_quality_score</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>defocus</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>astigmatism</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>wavenumber_min</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>wavenumber_max</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>spectral_resolution</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>number_of_scans</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>apodization_function</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>molecular_signatures</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>background_correction</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>excitation_wavelength</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>emission_wavelength</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>excitation_filter</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>emission_filter</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>fluorophore</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>channel_name</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>laser_power</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>pinhole_size</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>quantum_yield</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>defocus</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>astigmatism</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4977,7 +5222,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5106,7 +5351,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5132,7 +5377,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5183,7 +5428,38 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5219,7 +5495,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5255,59 +5531,28 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>attribute</t>
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>duration</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>temperature</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>duration</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
           <t>atmosphere</t>
         </is>
       </c>
@@ -5322,7 +5567,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5464,7 +5709,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5555,7 +5800,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5706,7 +5951,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5752,7 +5997,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5803,7 +6048,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5952,7 +6197,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5973,228 +6218,6 @@
         </is>
       </c>
       <c r="C1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AG1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>resolution</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>resolution_high_shell_a</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>resolution_low_a</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>completeness</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>completeness_high_res_shell_percent</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>signal_to_noise</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>mean_i_over_sigma_i</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>space_group</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>unit_cell_a</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>unit_cell_b</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>unit_cell_c</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>unit_cell_alpha</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>unit_cell_beta</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>unit_cell_gamma</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>multiplicity</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>cc_half</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>r_merge</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>r_pim</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>wilson_b_factor_a2</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>anomalous_used</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>anom_corr</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>anom_sig_ano</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>r_work</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>r_free</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>ramachandran_favored_percent</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>ramachandran_outliers_percent</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>clashscore</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>molprobity_score</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>average_b_factor_a2</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>i_zero</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>rg</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>r_factor</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>cpu_hours</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>gpu_hours</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>memory_gb</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>storage_gb</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -6297,6 +6320,228 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AG1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resolution</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>resolution_high_shell_a</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>resolution_low_a</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>completeness</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>completeness_high_res_shell_percent</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>signal_to_noise</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>mean_i_over_sigma_i</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>space_group</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>unit_cell_a</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>unit_cell_b</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>unit_cell_c</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>unit_cell_alpha</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>unit_cell_beta</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>unit_cell_gamma</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>multiplicity</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>cc_half</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>r_merge</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>r_pim</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>wilson_b_factor_a2</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>anomalous_used</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>anom_corr</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>anom_sig_ano</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>r_work</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>r_free</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>ramachandran_favored_percent</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>ramachandran_outliers_percent</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>clashscore</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>molprobity_score</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>average_b_factor_a2</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>i_zero</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>rg</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>r_factor</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>cpu_hours</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>gpu_hours</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>memory_gb</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>storage_gb</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -6352,7 +6597,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6403,7 +6648,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6464,7 +6709,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6530,7 +6775,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6561,7 +6806,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6602,7 +6847,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6628,7 +6873,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6654,7 +6899,133 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>site_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>site_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>residues</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ligand_interactions</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>conservation_score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>functional_importance</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>go_terms</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ec_number</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>protein_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pdb_entry</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>chain_id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>residue_range</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>confidence_score</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>evidence_type</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>evidence_code</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>source_database</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>annotation_method</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>publication_ids</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6695,7 +7066,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6731,133 +7102,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>site_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>site_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>residues</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>ligand_interactions</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>conservation_score</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>functional_importance</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>go_terms</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>ec_number</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>protein_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>pdb_entry</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>chain_id</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>residue_range</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>confidence_score</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>evidence_type</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>evidence_code</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>source_database</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>annotation_method</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>publication_ids</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6883,7 +7128,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6919,7 +7164,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6955,6 +7200,211 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>study_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>person_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>author_position</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>corresponding</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"principal_investigator,co_investigator,author,operator,local_contact,analyst,reviewer,data_curator,submitter,contact"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>experiment_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>person_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"principal_investigator,co_investigator,author,operator,local_contact,analyst,reviewer,data_curator,submitter,contact"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>workflow_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>person_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"principal_investigator,co_investigator,author,operator,local_contact,analyst,reviewer,data_curator,submitter,contact"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>study_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>award_number</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"host_institution,operating_institution,funder,collaborating_institution,depositor,primary_affiliation,secondary_affiliation,former_affiliation"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>person_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>organization_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"host_institution,operating_institution,funder,collaborating_institution,depositor,primary_affiliation,secondary_affiliation,former_affiliation"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Regenerate artifacts for the Protein entity
Turtle example outputs also change where blank nodes reorder; no content
differs there.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Syrj2YgvduteYzBeMfp8qf
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -31,62 +31,64 @@
     <sheet name="Person" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="Organization" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="Sample" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="ProteinConstruct" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="SamplePreparation" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Instrument" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="CryoEMInstrument" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="XRayInstrument" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="SANSDetector" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="SANSSource" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="SANSConfiguration" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="SANSInstrument" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="SAXSInstrument" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="BeamlineInstrument" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="ExperimentRun" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="WorkflowRun" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="DataFile" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="Image" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="Image2D" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="Image3D" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="Movie" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="Micrograph" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="FTIRImage" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="FluorescenceImage" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="OpticalImage" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="XRFImage" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="ImageFeature" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="OntologyTerm" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="MolecularComposition" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="BufferComposition" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="StorageConditions" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="CryoEMPreparation" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="CrystallizationConditions" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="XRayPreparation" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="SAXSPreparation" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="ExperimentalConditions" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="DataCollectionStrategy" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="BeamCenterPixels" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="QualityMetrics" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="ComputeResources" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="CryoEMQualityMetrics" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="MotionCorrectionParameters" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="CTFEstimationParameters" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="ParticlePickingParameters" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="RefinementParameters" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="FSCCurve" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="StudySampleAssociation" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="StudyExperimentAssociation" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="StudyWorkflowAssociation" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="ExperimentSampleAssociation" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="ExperimentInstrumentAssociation" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet name="WorkflowExperimentAssociation" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet name="WorkflowInputAssociation" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet name="WorkflowOutputAssociation" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet name="StudyPersonAssociation" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet name="ExperimentPersonAssociation" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet name="WorkflowPersonAssociation" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet name="StudyOrganizationAssociation" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet name="PersonOrganizationAssociation" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet name="Protein" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="ProteinConstruct" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="SamplePreparation" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Instrument" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="CryoEMInstrument" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="XRayInstrument" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="SANSDetector" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="SANSSource" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="SANSConfiguration" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="SANSInstrument" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="SAXSInstrument" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="BeamlineInstrument" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="ExperimentRun" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="WorkflowRun" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="DataFile" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="Image" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="Image2D" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="Image3D" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="Movie" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Micrograph" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="FTIRImage" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="FluorescenceImage" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="OpticalImage" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="XRFImage" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="ImageFeature" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="OntologyTerm" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="MolecularComposition" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="BufferComposition" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="StorageConditions" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="CryoEMPreparation" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="CrystallizationConditions" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="XRayPreparation" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="SAXSPreparation" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="ExperimentalConditions" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="DataCollectionStrategy" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="BeamCenterPixels" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="QualityMetrics" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="ComputeResources" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="CryoEMQualityMetrics" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="MotionCorrectionParameters" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="CTFEstimationParameters" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="ParticlePickingParameters" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="RefinementParameters" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="FSCCurve" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="StudySampleAssociation" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="StudyExperimentAssociation" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="StudyWorkflowAssociation" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="ExperimentSampleAssociation" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="SampleProteinAssociation" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="ExperimentInstrumentAssociation" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="WorkflowExperimentAssociation" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="WorkflowInputAssociation" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="WorkflowOutputAssociation" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="StudyPersonAssociation" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="ExperimentPersonAssociation" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet name="WorkflowPersonAssociation" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet name="StudyOrganizationAssociation" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet name="PersonOrganizationAssociation" sheetId="82" state="visible" r:id="rId82"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1452,7 +1454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AD1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1483,115 +1485,125 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>proteins</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>protein_constructs</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>samples</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>sample_preparations</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>experiment_runs</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>workflow_runs</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>data_files</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>images</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>study_sample_associations</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>study_experiment_associations</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>study_workflow_associations</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>experiment_sample_associations</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>experiment_instrument_associations</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>sample_protein_associations</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
         <is>
           <t>workflow_experiment_associations</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>workflow_input_associations</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>workflow_output_associations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>study_person_associations</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>experiment_person_associations</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>workflow_person_associations</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>study_organization_associations</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>person_organization_associations</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2013,7 +2025,148 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:Y1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>uniprot_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>protein_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>gene_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>organism</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>organism_name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>amino_acid_sequence</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sequence_length</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>molecular_weight_theoretical</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ec_numbers</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>function_description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>go_terms</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>pdb_entries</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>functional_sites</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>structural_features</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>protein_interactions</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>ligand_interactions</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>mutation_effects</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ptm_annotations</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>biophysical_properties</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>evolutionary_conservation</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>conformational_ensemble</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>cross_references</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2024,115 +2177,120 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>protein_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>uniprot_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>gene_name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>ncbi_taxid</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>sequence_length_aa</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>construct_description</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>gene_synthesis_provider</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>codon_optimization_organism</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>vector_backbone</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>vector_name</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>promoter</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>tag_nterm</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>tag_cterm</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>cleavage_site</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>signal_peptide</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>selectable_marker</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>cloning_method</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>insert_boundaries</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>sequence_file_path</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>sequence_verified_by</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>verification_notes</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2143,7 +2301,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2395,7 +2553,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2492,7 +2650,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2728,7 +2886,58 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>maximum_numeric_value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>minimum_numeric_value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>numeric_value</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>unit_cv_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2891,119 +3100,205 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>maximum_numeric_value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>minimum_numeric_value</t>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>detector_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>detector_type</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>numeric_value</t>
+          <t>detector_description</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>pixel_size_x</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>unit_cv_id</t>
+          <t>pixel_size_y</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>attribute</t>
+          <t>sample_detector_distance</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>detector_name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>detector_type</t>
+          <t>rotation_angle</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>beam_trap_type</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>beam_trap_position_x</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>beam_trap_position_y</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_description</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>detector_description</t>
+          <t>wavelength</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>pixel_size_x</t>
+          <t>wavelength_spread</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>pixel_size_y</t>
+          <t>wavelength_selection_method</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>sample_detector_distance</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>rotation_angle</t>
+          <t>flux</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>beam_trap_type</t>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>q_min</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>q_max</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>number_of_guides</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>attenuator</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>source_aperature_diameter</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sample_aperature_diameter</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>siwindow_to_main_distance</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>sample_ap_to_si_distance</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>beam_trap_position_x</t>
+          <t>sample_ap_to_main_distance</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>beam_trap_position_y</t>
+          <t>sample_ap_to_sample_distance</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>source_ap_to_siwindow_distance</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>source_ap_to_sample_ap_distance</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
@@ -3013,144 +3308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>wavelength</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>wavelength_spread</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>wavelength_selection_method</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>energy</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>flux</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>q_min</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>q_max</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>number_of_guides</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>attenuator</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>source_aperature_diameter</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>sample_aperature_diameter</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>siwindow_to_main_distance</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>sample_ap_to_si_distance</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>sample_ap_to_main_distance</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>sample_ap_to_sample_distance</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>source_ap_to_siwindow_distance</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>source_ap_to_sample_ap_distance</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3285,7 +3443,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3412,7 +3570,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3584,7 +3742,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3992,7 +4150,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4353,7 +4511,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4442,7 +4600,43 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value_cv_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4508,108 +4702,632 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>value_cv_id</t>
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>defocus</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>astigmatism</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>attribute</t>
+          <t>file_name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>dimensions_z</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>voxel_size</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>reconstruction_method</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AA1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>frames</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>super_resolution</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>pixel_size_unbinned</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>stage_position_x</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>stage_position_y</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>stage_position_z</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>nominal_defocus</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>dose_per_frame</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>beam_shift_x</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>beam_shift_y</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ice_thickness_estimate</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>grid_square_id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>hole_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>acquisition_group</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>defocus</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>astigmatism</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>origin_movie_id</t>
+        </is>
+      </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>defocus_u</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>defocus_v</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>astigmatism_angle</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>resolution_fit_limit</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ctf_quality_score</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>defocus</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>astigmatism</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>file_name</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>wavenumber_min</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>wavenumber_max</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>spectral_resolution</t>
+        </is>
+      </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>number_of_scans</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>apodization_function</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>molecular_signatures</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>background_correction</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>acquisition_date</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>excitation_wavelength</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>emission_wavelength</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>excitation_filter</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>emission_filter</t>
+        </is>
+      </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>fluorophore</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>channel_name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>laser_power</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>pinhole_size</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>quantum_yield</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>defocus</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>astigmatism</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>pixel_size</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dimensions_x</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>dimensions_y</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>exposure_time</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>dose</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -4620,567 +5338,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>dimensions_z</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>voxel_size</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>reconstruction_method</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AA1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>frames</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>super_resolution</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>pixel_size_unbinned</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>stage_position_x</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>stage_position_y</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>stage_position_z</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>nominal_defocus</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>dose_per_frame</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>beam_shift_x</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>beam_shift_y</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>ice_thickness_estimate</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>grid_square_id</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>hole_id</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>acquisition_group</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>defocus</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>astigmatism</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:R1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>origin_movie_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>defocus_u</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>defocus_v</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>astigmatism_angle</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>resolution_fit_limit</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>ctf_quality_score</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>defocus</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>astigmatism</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>wavenumber_min</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>wavenumber_max</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>spectral_resolution</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>number_of_scans</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>apodization_function</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>molecular_signatures</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>background_correction</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>excitation_wavelength</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>emission_wavelength</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>excitation_filter</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>emission_filter</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>fluorophore</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>channel_name</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>laser_power</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>pinhole_size</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>quantum_yield</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>defocus</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>astigmatism</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5291,7 +5449,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5420,7 +5578,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5446,7 +5604,38 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5497,38 +5686,43 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>attribute</t>
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sequences</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>modifications</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>ligands</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5540,17 +5734,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>sequences</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>modifications</t>
+          <t>ph</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>components</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>ligands</t>
+          <t>additives</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -5564,7 +5758,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5576,17 +5770,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ph</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>components</t>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>duration</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>additives</t>
+          <t>atmosphere</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -5600,43 +5794,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>temperature</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>duration</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>atmosphere</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5778,7 +5936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5869,7 +6027,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6020,7 +6178,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6066,7 +6224,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6117,7 +6275,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6266,37 +6424,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>xbeam</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>ybeam</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -6389,6 +6516,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>xbeam</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ybeam</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AH1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -6569,7 +6727,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6610,7 +6768,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6657,7 +6815,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6718,7 +6876,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6769,7 +6927,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6830,7 +6988,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6896,7 +7054,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6927,7 +7085,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6968,32 +7126,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>study_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>experiment_id</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7137,6 +7269,32 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>experiment_id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>study_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>workflow_id</t>
         </is>
       </c>
@@ -7146,7 +7304,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7187,7 +7345,78 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sample_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>protein_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>construct_id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>copy_number</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>residue_range</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sequence_coverage</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>chain_ids</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>modifications</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>observed_molecular_weight</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"target,subunit,binding_partner,fusion_partner,chaperone,contaminant,standard"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7223,7 +7452,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7249,7 +7478,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7285,7 +7514,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7321,7 +7550,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7367,7 +7596,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7403,7 +7632,147 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>feature_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>secondary_structure</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>solvent_accessibility</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>backbone_flexibility</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>disorder_probability</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>conformational_state</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>structural_motif</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>domain_assignment</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>domain_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>protein_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>pdb_entry</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>chain_id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>residue_range</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>confidence_score</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>evidence_type</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>evidence_code</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>source_database</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>annotation_method</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>publication_ids</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"alpha_helix,beta_sheet,beta_strand,turn,coil,disordered_region,transmembrane_helix,signal_peptide,transit_peptide,domain,repeat,zinc_finger,zinc_binding,coiled_coil,motif,cavity,channel,pore,hinge,linker"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"helix,sheet,turn,coil,helix_310,helix_pi,bend,bridge"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"open,closed,intermediate,active,inactive,apo,holo,substrate_bound,product_bound,inhibitor_bound,partially_open,partially_closed,disordered"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7439,7 +7808,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7480,147 +7849,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:V1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>feature_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>secondary_structure</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>solvent_accessibility</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>backbone_flexibility</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>disorder_probability</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>conformational_state</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>structural_motif</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>domain_assignment</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>domain_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>protein_id</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>pdb_entry</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>chain_id</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>residue_range</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>confidence_score</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>evidence_type</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>evidence_code</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>source_database</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>annotation_method</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>publication_ids</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"alpha_helix,beta_sheet,beta_strand,turn,coil,disordered_region,transmembrane_helix,signal_peptide,transit_peptide,domain,repeat,zinc_finger,zinc_binding,coiled_coil,motif,cavity,channel,pore,hinge,linker"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"helix,sheet,turn,coil,helix_310,helix_pi,bend,bridge"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"open,closed,intermediate,active,inactive,apo,holo,substrate_bound,product_bound,inhibitor_bound,partially_open,partially_closed,disordered"</formula1>
-    </dataValidation>
-    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>